<commit_message>
Add Terminated and Retired employees to sample data
Sample data only had Resigned leavers, so Overall Turnover and
Attrition showed the same value. Reassigned some leavers to
Terminated and Retired (older employees) so the two metrics differ.
</commit_message>
<xml_diff>
--- a/documents/customer_support.xlsx
+++ b/documents/customer_support.xlsx
@@ -516,7 +516,6 @@
           <t>2022-03-28</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>54200</v>
       </c>
@@ -568,7 +567,6 @@
           <t>2021-05-13</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
         <v>80500</v>
       </c>
@@ -620,7 +618,6 @@
           <t>2022-02-22</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
         <v>58200</v>
       </c>
@@ -672,7 +669,6 @@
           <t>2024-05-27</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
         <v>76200</v>
       </c>
@@ -724,7 +720,6 @@
           <t>2024-01-27</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
         <v>70300</v>
       </c>
@@ -776,7 +771,6 @@
           <t>2019-07-14</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
         <v>60700</v>
       </c>
@@ -828,7 +822,6 @@
           <t>2022-01-20</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
         <v>79200</v>
       </c>
@@ -880,7 +873,6 @@
           <t>2026-02-25</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
         <v>67500</v>
       </c>
@@ -932,7 +924,6 @@
           <t>2024-05-24</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
         <v>54500</v>
       </c>
@@ -984,7 +975,6 @@
           <t>2024-07-20</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
         <v>76300</v>
       </c>
@@ -1036,7 +1026,6 @@
           <t>2021-06-09</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
         <v>64100</v>
       </c>
@@ -1088,7 +1077,6 @@
           <t>2023-02-08</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
         <v>54400</v>
       </c>
@@ -1140,7 +1128,6 @@
           <t>2023-08-14</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
         <v>77300</v>
       </c>
@@ -1192,7 +1179,6 @@
           <t>2022-09-18</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
         <v>75200</v>
       </c>
@@ -1244,7 +1230,6 @@
           <t>2026-04-14</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
         <v>47900</v>
       </c>
@@ -1296,7 +1281,6 @@
           <t>2023-10-20</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
         <v>56800</v>
       </c>
@@ -1348,7 +1332,6 @@
           <t>2023-05-15</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="n">
         <v>66700</v>
       </c>
@@ -1400,7 +1383,6 @@
           <t>2021-05-05</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
       <c r="G19" t="n">
         <v>56800</v>
       </c>
@@ -1452,7 +1434,6 @@
           <t>2023-06-24</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="n">
         <v>70700</v>
       </c>
@@ -1504,7 +1485,6 @@
           <t>2024-07-05</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
       <c r="G21" t="n">
         <v>50800</v>
       </c>
@@ -1556,7 +1536,6 @@
           <t>2022-12-26</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
       <c r="G22" t="n">
         <v>50300</v>
       </c>
@@ -1608,7 +1587,6 @@
           <t>2025-09-17</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
       <c r="G23" t="n">
         <v>52600</v>
       </c>
@@ -1660,7 +1638,6 @@
           <t>2023-09-05</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="n">
         <v>66300</v>
       </c>
@@ -1712,7 +1689,6 @@
           <t>2023-07-15</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
       <c r="G25" t="n">
         <v>52000</v>
       </c>
@@ -1764,7 +1740,6 @@
           <t>2024-09-09</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
       <c r="G26" t="n">
         <v>50400</v>
       </c>
@@ -1816,7 +1791,6 @@
           <t>2024-05-11</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
       <c r="G27" t="n">
         <v>48800</v>
       </c>
@@ -1868,7 +1842,6 @@
           <t>2022-03-07</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
       <c r="G28" t="n">
         <v>58700</v>
       </c>
@@ -1920,7 +1893,6 @@
           <t>2025-07-01</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
       <c r="G29" t="n">
         <v>66500</v>
       </c>
@@ -1972,7 +1944,6 @@
           <t>2023-01-13</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
       <c r="G30" t="n">
         <v>50200</v>
       </c>
@@ -2024,7 +1995,6 @@
           <t>2025-05-11</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
       <c r="G31" t="n">
         <v>56900</v>
       </c>
@@ -2076,7 +2046,6 @@
           <t>2023-10-02</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="n">
         <v>51700</v>
       </c>
@@ -2128,7 +2097,6 @@
           <t>2024-04-17</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" t="n">
         <v>60400</v>
       </c>
@@ -2180,7 +2148,6 @@
           <t>2023-11-04</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" t="n">
         <v>51800</v>
       </c>
@@ -2232,7 +2199,6 @@
           <t>2023-01-25</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
       <c r="G35" t="n">
         <v>83100</v>
       </c>
@@ -2284,7 +2250,6 @@
           <t>2023-08-16</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
       <c r="G36" t="n">
         <v>52900</v>
       </c>
@@ -2336,7 +2301,6 @@
           <t>2025-11-08</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
       <c r="G37" t="n">
         <v>65800</v>
       </c>
@@ -2388,7 +2352,6 @@
           <t>2022-10-08</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
       <c r="G38" t="n">
         <v>66800</v>
       </c>
@@ -2440,7 +2403,6 @@
           <t>2026-04-03</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
       <c r="G39" t="n">
         <v>62600</v>
       </c>
@@ -2492,7 +2454,6 @@
           <t>2025-05-03</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
       <c r="G40" t="n">
         <v>64200</v>
       </c>
@@ -2544,7 +2505,6 @@
           <t>2024-01-06</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
       <c r="G41" t="n">
         <v>56300</v>
       </c>
@@ -2596,7 +2556,6 @@
           <t>2025-02-12</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
       <c r="G42" t="n">
         <v>61400</v>
       </c>
@@ -2648,7 +2607,6 @@
           <t>2023-04-24</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
       <c r="G43" t="n">
         <v>51800</v>
       </c>
@@ -2700,7 +2658,6 @@
           <t>2023-06-17</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
       <c r="G44" t="n">
         <v>87500</v>
       </c>
@@ -2752,7 +2709,6 @@
           <t>2019-06-01</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
       <c r="G45" t="n">
         <v>96000</v>
       </c>
@@ -2804,7 +2760,6 @@
           <t>2025-08-09</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
       <c r="G46" t="n">
         <v>50500</v>
       </c>
@@ -2856,7 +2811,6 @@
           <t>2024-03-09</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
       <c r="G47" t="n">
         <v>86700</v>
       </c>
@@ -2908,7 +2862,6 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
       <c r="G48" t="n">
         <v>53800</v>
       </c>
@@ -2960,7 +2913,6 @@
           <t>2023-10-12</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
       <c r="G49" t="n">
         <v>58100</v>
       </c>
@@ -3012,7 +2964,6 @@
           <t>2022-07-08</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
       <c r="G50" t="n">
         <v>61600</v>
       </c>
@@ -3064,7 +3015,6 @@
           <t>2022-09-02</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
       <c r="G51" t="n">
         <v>69000</v>
       </c>
@@ -3116,7 +3066,6 @@
           <t>2022-05-15</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
       <c r="G52" t="n">
         <v>52300</v>
       </c>
@@ -3168,7 +3117,6 @@
           <t>2022-11-17</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
       <c r="G53" t="n">
         <v>53600</v>
       </c>
@@ -3220,7 +3168,6 @@
           <t>2019-08-26</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
       <c r="G54" t="n">
         <v>72800</v>
       </c>
@@ -3272,7 +3219,6 @@
           <t>2024-01-12</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
       <c r="G55" t="n">
         <v>100800</v>
       </c>
@@ -3324,7 +3270,6 @@
           <t>2025-11-04</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
       <c r="G56" t="n">
         <v>47600</v>
       </c>
@@ -3376,7 +3321,6 @@
           <t>2023-12-19</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
       <c r="G57" t="n">
         <v>59600</v>
       </c>
@@ -3428,7 +3372,6 @@
           <t>2024-05-13</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
       <c r="G58" t="n">
         <v>62800</v>
       </c>
@@ -3480,7 +3423,6 @@
           <t>2022-10-28</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
       <c r="G59" t="n">
         <v>52500</v>
       </c>
@@ -3532,7 +3474,6 @@
           <t>2019-12-17</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
       <c r="G60" t="n">
         <v>70300</v>
       </c>
@@ -3584,7 +3525,6 @@
           <t>2023-02-18</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
       <c r="G61" t="n">
         <v>51900</v>
       </c>
@@ -3636,7 +3576,6 @@
           <t>2023-06-12</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
       <c r="G62" t="n">
         <v>52500</v>
       </c>
@@ -3688,7 +3627,6 @@
           <t>2024-05-10</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
       <c r="G63" t="n">
         <v>66200</v>
       </c>
@@ -3740,7 +3678,6 @@
           <t>2022-09-23</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
       <c r="G64" t="n">
         <v>60600</v>
       </c>
@@ -3792,7 +3729,6 @@
           <t>2021-01-09</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
       <c r="G65" t="n">
         <v>67900</v>
       </c>
@@ -3844,7 +3780,6 @@
           <t>2022-10-02</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
       <c r="G66" t="n">
         <v>52000</v>
       </c>
@@ -3896,7 +3831,6 @@
           <t>2024-12-14</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
       <c r="G67" t="n">
         <v>57300</v>
       </c>
@@ -3948,7 +3882,6 @@
           <t>2022-06-16</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr"/>
       <c r="G68" t="n">
         <v>53900</v>
       </c>
@@ -4000,7 +3933,6 @@
           <t>2019-08-14</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr"/>
       <c r="G69" t="n">
         <v>98000</v>
       </c>
@@ -4052,7 +3984,6 @@
           <t>2022-11-10</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
       <c r="G70" t="n">
         <v>72300</v>
       </c>
@@ -4104,7 +4035,6 @@
           <t>2023-01-01</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
       <c r="G71" t="n">
         <v>61400</v>
       </c>
@@ -4156,7 +4086,6 @@
           <t>2025-11-24</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr"/>
       <c r="G72" t="n">
         <v>67900</v>
       </c>
@@ -4208,7 +4137,6 @@
           <t>2020-04-09</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
       <c r="G73" t="n">
         <v>53600</v>
       </c>
@@ -4260,7 +4188,6 @@
           <t>2024-12-19</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr"/>
       <c r="G74" t="n">
         <v>70300</v>
       </c>
@@ -4312,7 +4239,6 @@
           <t>2024-11-28</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
       <c r="G75" t="n">
         <v>57200</v>
       </c>
@@ -4364,7 +4290,6 @@
           <t>2019-06-25</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr"/>
       <c r="G76" t="n">
         <v>92000</v>
       </c>
@@ -4416,7 +4341,6 @@
           <t>2021-09-11</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
       <c r="G77" t="n">
         <v>73000</v>
       </c>
@@ -4468,7 +4392,6 @@
           <t>2024-09-21</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
       <c r="G78" t="n">
         <v>83000</v>
       </c>
@@ -4520,7 +4443,6 @@
           <t>2023-09-05</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr"/>
       <c r="G79" t="n">
         <v>51300</v>
       </c>
@@ -4572,7 +4494,6 @@
           <t>2025-03-05</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr"/>
       <c r="G80" t="n">
         <v>48400</v>
       </c>
@@ -4624,7 +4545,6 @@
           <t>2023-11-03</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr"/>
       <c r="G81" t="n">
         <v>63400</v>
       </c>
@@ -4676,7 +4596,6 @@
           <t>2025-12-11</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr"/>
       <c r="G82" t="n">
         <v>77200</v>
       </c>
@@ -4728,7 +4647,6 @@
           <t>2023-10-19</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
       <c r="G83" t="n">
         <v>95800</v>
       </c>
@@ -4780,7 +4698,6 @@
           <t>2024-08-01</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr"/>
       <c r="G84" t="n">
         <v>76000</v>
       </c>
@@ -4832,7 +4749,6 @@
           <t>2024-12-22</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr"/>
       <c r="G85" t="n">
         <v>61800</v>
       </c>
@@ -4884,7 +4800,6 @@
           <t>2024-03-25</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr"/>
       <c r="G86" t="n">
         <v>50500</v>
       </c>
@@ -4936,7 +4851,6 @@
           <t>2023-07-14</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr"/>
       <c r="G87" t="n">
         <v>67200</v>
       </c>
@@ -4988,7 +4902,6 @@
           <t>2022-11-12</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr"/>
       <c r="G88" t="n">
         <v>61000</v>
       </c>
@@ -5040,7 +4953,6 @@
           <t>2025-08-20</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr"/>
       <c r="G89" t="n">
         <v>55600</v>
       </c>
@@ -5092,7 +5004,6 @@
           <t>2025-07-04</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr"/>
       <c r="G90" t="n">
         <v>75100</v>
       </c>
@@ -5144,7 +5055,6 @@
           <t>2024-04-07</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr"/>
       <c r="G91" t="n">
         <v>52500</v>
       </c>
@@ -5196,7 +5106,6 @@
           <t>2019-03-26</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr"/>
       <c r="G92" t="n">
         <v>80300</v>
       </c>
@@ -5248,7 +5157,6 @@
           <t>2024-08-20</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr"/>
       <c r="G93" t="n">
         <v>52000</v>
       </c>
@@ -5300,7 +5208,6 @@
           <t>2024-02-24</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr"/>
       <c r="G94" t="n">
         <v>61200</v>
       </c>
@@ -5352,7 +5259,6 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr"/>
       <c r="G95" t="n">
         <v>54000</v>
       </c>
@@ -5404,7 +5310,6 @@
           <t>2024-04-21</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
       <c r="G96" t="n">
         <v>63800</v>
       </c>
@@ -5456,7 +5361,6 @@
           <t>2026-03-28</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr"/>
       <c r="G97" t="n">
         <v>60900</v>
       </c>
@@ -5508,7 +5412,6 @@
           <t>2024-01-21</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr"/>
       <c r="G98" t="n">
         <v>56300</v>
       </c>
@@ -5560,7 +5463,6 @@
           <t>2024-06-07</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr"/>
       <c r="G99" t="n">
         <v>94900</v>
       </c>
@@ -5612,7 +5514,6 @@
           <t>2025-09-08</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr"/>
       <c r="G100" t="n">
         <v>81800</v>
       </c>
@@ -5664,7 +5565,6 @@
           <t>2023-12-19</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr"/>
       <c r="G101" t="n">
         <v>82500</v>
       </c>
@@ -5716,7 +5616,6 @@
           <t>2024-03-16</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr"/>
       <c r="G102" t="n">
         <v>86300</v>
       </c>
@@ -5768,7 +5667,6 @@
           <t>2022-11-09</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr"/>
       <c r="G103" t="n">
         <v>80500</v>
       </c>
@@ -5820,7 +5718,6 @@
           <t>2022-01-19</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr"/>
       <c r="G104" t="n">
         <v>88100</v>
       </c>
@@ -5872,7 +5769,6 @@
           <t>2024-05-18</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr"/>
       <c r="G105" t="n">
         <v>61700</v>
       </c>
@@ -5924,7 +5820,6 @@
           <t>2024-01-27</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr"/>
       <c r="G106" t="n">
         <v>80200</v>
       </c>
@@ -5976,7 +5871,6 @@
           <t>2023-12-18</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr"/>
       <c r="G107" t="n">
         <v>64700</v>
       </c>
@@ -6028,7 +5922,6 @@
           <t>2024-09-03</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr"/>
       <c r="G108" t="n">
         <v>83500</v>
       </c>
@@ -6080,7 +5973,6 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr"/>
       <c r="G109" t="n">
         <v>51100</v>
       </c>
@@ -6132,7 +6024,6 @@
           <t>2024-10-26</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr"/>
       <c r="G110" t="n">
         <v>49900</v>
       </c>
@@ -6184,7 +6075,6 @@
           <t>2022-06-25</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr"/>
       <c r="G111" t="n">
         <v>74100</v>
       </c>
@@ -6236,7 +6126,6 @@
           <t>2024-08-06</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr"/>
       <c r="G112" t="n">
         <v>71600</v>
       </c>
@@ -6288,7 +6177,6 @@
           <t>2022-03-24</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr"/>
       <c r="G113" t="n">
         <v>61400</v>
       </c>
@@ -6340,7 +6228,6 @@
           <t>2021-08-19</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr"/>
       <c r="G114" t="n">
         <v>50300</v>
       </c>
@@ -6392,7 +6279,6 @@
           <t>2023-01-03</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr"/>
       <c r="G115" t="n">
         <v>87500</v>
       </c>
@@ -6444,7 +6330,6 @@
           <t>2024-10-04</t>
         </is>
       </c>
-      <c r="F116" t="inlineStr"/>
       <c r="G116" t="n">
         <v>52600</v>
       </c>
@@ -6496,7 +6381,6 @@
           <t>2022-10-05</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr"/>
       <c r="G117" t="n">
         <v>53500</v>
       </c>
@@ -6548,7 +6432,6 @@
           <t>2024-03-11</t>
         </is>
       </c>
-      <c r="F118" t="inlineStr"/>
       <c r="G118" t="n">
         <v>70500</v>
       </c>
@@ -6600,7 +6483,6 @@
           <t>2024-10-01</t>
         </is>
       </c>
-      <c r="F119" t="inlineStr"/>
       <c r="G119" t="n">
         <v>55700</v>
       </c>
@@ -6652,7 +6534,6 @@
           <t>2023-07-13</t>
         </is>
       </c>
-      <c r="F120" t="inlineStr"/>
       <c r="G120" t="n">
         <v>72600</v>
       </c>
@@ -6704,7 +6585,6 @@
           <t>2022-07-15</t>
         </is>
       </c>
-      <c r="F121" t="inlineStr"/>
       <c r="G121" t="n">
         <v>76300</v>
       </c>
@@ -6756,7 +6636,6 @@
           <t>2019-10-03</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr"/>
       <c r="G122" t="n">
         <v>64200</v>
       </c>
@@ -6808,7 +6687,6 @@
           <t>2024-08-10</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr"/>
       <c r="G123" t="n">
         <v>56400</v>
       </c>
@@ -6860,7 +6738,6 @@
           <t>2024-11-24</t>
         </is>
       </c>
-      <c r="F124" t="inlineStr"/>
       <c r="G124" t="n">
         <v>95100</v>
       </c>
@@ -6912,7 +6789,6 @@
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="F125" t="inlineStr"/>
       <c r="G125" t="n">
         <v>62800</v>
       </c>
@@ -6964,7 +6840,6 @@
           <t>2023-10-16</t>
         </is>
       </c>
-      <c r="F126" t="inlineStr"/>
       <c r="G126" t="n">
         <v>60000</v>
       </c>
@@ -7016,7 +6891,6 @@
           <t>2023-12-21</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr"/>
       <c r="G127" t="n">
         <v>46700</v>
       </c>
@@ -7068,7 +6942,6 @@
           <t>2023-01-23</t>
         </is>
       </c>
-      <c r="F128" t="inlineStr"/>
       <c r="G128" t="n">
         <v>56700</v>
       </c>
@@ -7120,7 +6993,6 @@
           <t>2023-05-17</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr"/>
       <c r="G129" t="n">
         <v>60000</v>
       </c>
@@ -7172,7 +7044,6 @@
           <t>2019-04-12</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr"/>
       <c r="G130" t="n">
         <v>62900</v>
       </c>
@@ -7224,7 +7095,6 @@
           <t>2023-03-19</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr"/>
       <c r="G131" t="n">
         <v>88000</v>
       </c>
@@ -7444,7 +7314,6 @@
           <t>2024-02-21</t>
         </is>
       </c>
-      <c r="F135" t="inlineStr"/>
       <c r="G135" t="n">
         <v>61900</v>
       </c>
@@ -7506,7 +7375,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I136" t="n">
@@ -7730,7 +7599,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Retired</t>
         </is>
       </c>
       <c r="I140" t="n">
@@ -7842,7 +7711,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I142" t="n">
@@ -8010,7 +7879,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I145" t="n">
@@ -8178,7 +8047,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I148" t="n">
@@ -8514,7 +8383,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I154" t="n">
@@ -8794,7 +8663,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I159" t="n">
@@ -9298,7 +9167,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I168" t="n">
@@ -9578,7 +9447,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I173" t="n">
@@ -9858,7 +9727,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I178" t="n">
@@ -9914,7 +9783,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I179" t="n">
@@ -9970,7 +9839,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I180" t="n">
@@ -10026,7 +9895,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I181" t="n">
@@ -10082,7 +9951,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I182" t="n">
@@ -10194,7 +10063,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I184" t="n">
@@ -10250,7 +10119,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I185" t="n">
@@ -10922,7 +10791,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I197" t="n">
@@ -11090,7 +10959,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I200" t="n">
@@ -11426,7 +11295,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I206" t="n">
@@ -11594,7 +11463,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I209" t="n">
@@ -12154,7 +12023,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I219" t="n">
@@ -12378,7 +12247,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I223" t="n">
@@ -12546,7 +12415,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I226" t="n">
@@ -13442,7 +13311,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I242" t="n">
@@ -13890,7 +13759,7 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I250" t="n">
@@ -13946,7 +13815,7 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I251" t="n">
@@ -14002,7 +13871,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I252" t="n">
@@ -14058,7 +13927,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I253" t="n">
@@ -14282,7 +14151,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I257" t="n">
@@ -14394,7 +14263,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I259" t="n">
@@ -14506,7 +14375,7 @@
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I261" t="n">
@@ -15504,7 +15373,6 @@
           <t>2024-01-05</t>
         </is>
       </c>
-      <c r="F279" t="inlineStr"/>
       <c r="G279" t="n">
         <v>61400</v>
       </c>
@@ -15846,7 +15714,7 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I285" t="n">
@@ -16910,7 +16778,7 @@
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I304" t="n">
@@ -16966,7 +16834,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I305" t="n">
@@ -17302,7 +17170,7 @@
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I311" t="n">
@@ -17414,7 +17282,7 @@
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I313" t="n">
@@ -17572,7 +17440,6 @@
           <t>2023-10-03</t>
         </is>
       </c>
-      <c r="F316" t="inlineStr"/>
       <c r="G316" t="n">
         <v>51000</v>
       </c>
@@ -17634,7 +17501,7 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I317" t="n">
@@ -17690,7 +17557,7 @@
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I318" t="n">
@@ -17802,7 +17669,7 @@
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I320" t="n">
@@ -17914,7 +17781,7 @@
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I322" t="n">
@@ -18138,7 +18005,7 @@
       </c>
       <c r="H326" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I326" t="n">
@@ -18306,7 +18173,7 @@
       </c>
       <c r="H329" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I329" t="n">
@@ -18362,7 +18229,7 @@
       </c>
       <c r="H330" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I330" t="n">
@@ -18530,7 +18397,7 @@
       </c>
       <c r="H333" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I333" t="n">
@@ -18586,7 +18453,7 @@
       </c>
       <c r="H334" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I334" t="n">
@@ -19146,7 +19013,7 @@
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I344" t="n">
@@ -19314,7 +19181,7 @@
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I347" t="n">
@@ -19706,7 +19573,7 @@
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I354" t="n">
@@ -19920,7 +19787,6 @@
           <t>2022-07-06</t>
         </is>
       </c>
-      <c r="F358" t="inlineStr"/>
       <c r="G358" t="n">
         <v>58000</v>
       </c>
@@ -19982,7 +19848,7 @@
       </c>
       <c r="H359" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I359" t="n">
@@ -20206,7 +20072,7 @@
       </c>
       <c r="H363" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I363" t="n">
@@ -20374,7 +20240,7 @@
       </c>
       <c r="H366" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I366" t="n">
@@ -20486,7 +20352,7 @@
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I368" t="n">
@@ -20654,7 +20520,7 @@
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I371" t="n">
@@ -20700,7 +20566,6 @@
           <t>2022-12-16</t>
         </is>
       </c>
-      <c r="F372" t="inlineStr"/>
       <c r="G372" t="n">
         <v>51700</v>
       </c>
@@ -21042,7 +20907,7 @@
       </c>
       <c r="H378" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I378" t="n">
@@ -21378,7 +21243,7 @@
       </c>
       <c r="H384" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I384" t="n">
@@ -21490,7 +21355,7 @@
       </c>
       <c r="H386" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I386" t="n">
@@ -21994,7 +21859,7 @@
       </c>
       <c r="H395" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I395" t="n">
@@ -22050,7 +21915,7 @@
       </c>
       <c r="H396" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I396" t="n">
@@ -22274,7 +22139,7 @@
       </c>
       <c r="H400" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I400" t="n">
@@ -22834,7 +22699,7 @@
       </c>
       <c r="H410" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I410" t="n">
@@ -22890,7 +22755,7 @@
       </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I411" t="n">
@@ -23058,7 +22923,7 @@
       </c>
       <c r="H414" t="inlineStr">
         <is>
-          <t>Resigned</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I414" t="n">

</xml_diff>

<commit_message>
Extend sample data to October 2026
Sample data stopped in April 2026, so time-series charts and forecasts
dropped to zero for recent months. Added new hires (May-Oct) and
leavers (Apr-Oct) at the same rates as the previous year, in every
sample CSV/XLSX file.
</commit_message>
<xml_diff>
--- a/documents/customer_support.xlsx
+++ b/documents/customer_support.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L419"/>
+  <dimension ref="A1:L428"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -669,12 +669,17 @@
           <t>2024-05-27</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="G5" t="n">
         <v>76200</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -924,12 +929,17 @@
           <t>2024-05-24</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
       <c r="G10" t="n">
         <v>54500</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -1077,12 +1087,17 @@
           <t>2023-02-08</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
       <c r="G13" t="n">
         <v>54400</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -1434,12 +1449,17 @@
           <t>2023-06-24</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
       <c r="G20" t="n">
         <v>70700</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I20" t="n">
@@ -1485,12 +1505,17 @@
           <t>2024-07-05</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
       <c r="G21" t="n">
         <v>50800</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I21" t="n">
@@ -1842,12 +1867,17 @@
           <t>2022-03-07</t>
         </is>
       </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="G28" t="n">
         <v>58700</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I28" t="n">
@@ -1944,12 +1974,17 @@
           <t>2023-01-13</t>
         </is>
       </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
       <c r="G30" t="n">
         <v>50200</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I30" t="n">
@@ -1995,12 +2030,17 @@
           <t>2025-05-11</t>
         </is>
       </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="G31" t="n">
         <v>56900</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I31" t="n">
@@ -2148,12 +2188,17 @@
           <t>2023-11-04</t>
         </is>
       </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
       <c r="G34" t="n">
         <v>51800</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I34" t="n">
@@ -2199,12 +2244,17 @@
           <t>2023-01-25</t>
         </is>
       </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
       <c r="G35" t="n">
         <v>83100</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I35" t="n">
@@ -2607,12 +2657,17 @@
           <t>2023-04-24</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
       <c r="G43" t="n">
         <v>51800</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I43" t="n">
@@ -2964,12 +3019,17 @@
           <t>2022-07-08</t>
         </is>
       </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
       <c r="G50" t="n">
         <v>61600</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I50" t="n">
@@ -3321,12 +3381,17 @@
           <t>2023-12-19</t>
         </is>
       </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
       <c r="G57" t="n">
         <v>59600</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I57" t="n">
@@ -3474,12 +3539,17 @@
           <t>2019-12-17</t>
         </is>
       </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
       <c r="G60" t="n">
         <v>70300</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I60" t="n">
@@ -3525,12 +3595,17 @@
           <t>2023-02-18</t>
         </is>
       </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
       <c r="G61" t="n">
         <v>51900</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I61" t="n">
@@ -3729,12 +3804,17 @@
           <t>2021-01-09</t>
         </is>
       </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
       <c r="G65" t="n">
         <v>67900</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I65" t="n">
@@ -4239,12 +4319,17 @@
           <t>2024-11-28</t>
         </is>
       </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
       <c r="G75" t="n">
         <v>57200</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I75" t="n">
@@ -4290,12 +4375,17 @@
           <t>2019-06-25</t>
         </is>
       </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
       <c r="G76" t="n">
         <v>92000</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I76" t="n">
@@ -5106,12 +5196,17 @@
           <t>2019-03-26</t>
         </is>
       </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
       <c r="G92" t="n">
         <v>80300</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I92" t="n">
@@ -5157,12 +5252,17 @@
           <t>2024-08-20</t>
         </is>
       </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="G93" t="n">
         <v>52000</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I93" t="n">
@@ -5667,12 +5767,17 @@
           <t>2022-11-09</t>
         </is>
       </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
       <c r="G103" t="n">
         <v>80500</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I103" t="n">
@@ -6177,12 +6282,17 @@
           <t>2022-03-24</t>
         </is>
       </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
       <c r="G113" t="n">
         <v>61400</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I113" t="n">
@@ -6687,12 +6797,17 @@
           <t>2024-08-10</t>
         </is>
       </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
       <c r="G123" t="n">
         <v>56400</v>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Resigned</t>
         </is>
       </c>
       <c r="I123" t="n">
@@ -6789,12 +6904,17 @@
           <t>2026-03-05</t>
         </is>
       </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
       <c r="G125" t="n">
         <v>62800</v>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I125" t="n">
@@ -6891,12 +7011,17 @@
           <t>2023-12-21</t>
         </is>
       </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="G127" t="n">
         <v>46700</v>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Terminated</t>
         </is>
       </c>
       <c r="I127" t="n">
@@ -23220,6 +23345,465 @@
       <c r="L419" t="inlineStr">
         <is>
           <t>Hispanic</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>Angela Bailey</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>2003-09-14</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Customer Support</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Senior Support Agent</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="G420" t="n">
+        <v>61800</v>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I420" t="n">
+        <v>3</v>
+      </c>
+      <c r="J420" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K420" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="L420" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>Sara Torres</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>1976-11-18</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Customer Support</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Senior Support Agent</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="G421" t="n">
+        <v>56300</v>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I421" t="n">
+        <v>3</v>
+      </c>
+      <c r="J421" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="K421" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="L421" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>Diana Long</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>2001-05-25</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Customer Support</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Senior Support Agent</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="G422" t="n">
+        <v>64700</v>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I422" t="n">
+        <v>0</v>
+      </c>
+      <c r="J422" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="K422" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L422" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Douglas Henderson</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>2001-01-28</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Customer Support</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Team Lead</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="G423" t="n">
+        <v>80100</v>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I423" t="n">
+        <v>0</v>
+      </c>
+      <c r="J423" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="K423" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L423" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>William Ramirez</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>1993-01-14</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Customer Support</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Team Lead</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="G424" t="n">
+        <v>85800</v>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I424" t="n">
+        <v>2</v>
+      </c>
+      <c r="J424" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K424" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L424" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>Heather Anderson</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>1997-04-29</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Customer Support</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Senior Support Agent</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="G425" t="n">
+        <v>62800</v>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I425" t="n">
+        <v>2</v>
+      </c>
+      <c r="J425" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="K425" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="L425" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>Alan Ortiz</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>1986-07-24</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Customer Support</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Team Lead</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="G426" t="n">
+        <v>75200</v>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I426" t="n">
+        <v>3</v>
+      </c>
+      <c r="J426" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="K426" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L426" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>Joshua Kelly</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>1981-04-21</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Customer Support</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Senior Support Agent</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="G427" t="n">
+        <v>60400</v>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I427" t="n">
+        <v>2</v>
+      </c>
+      <c r="J427" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="K427" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="L427" t="inlineStr">
+        <is>
+          <t>Asian</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>Zachary Perry</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>1990-05-15</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Customer Support</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Team Lead</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="G428" t="n">
+        <v>94600</v>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I428" t="n">
+        <v>3</v>
+      </c>
+      <c r="J428" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="K428" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t>White</t>
         </is>
       </c>
     </row>

</xml_diff>